<commit_message>
feat(analytics): eliminate zero flatlines with continuous 245-day active consumption and balanced replenishments
</commit_message>
<xml_diff>
--- a/RMIMS_59_RAW_MATERIALS_CATALOG.xlsx
+++ b/RMIMS_59_RAW_MATERIALS_CATALOG.xlsx
@@ -429,12 +429,12 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>category</t>
+          <t>unit_of_measure</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>unit_of_measure</t>
+          <t>current_stock</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
@@ -454,7 +454,7 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>initial_stock</t>
+          <t>shortage_status</t>
         </is>
       </c>
     </row>
@@ -466,30 +466,30 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Food Grade Sunset Yellow / Orange Dye</t>
+          <t>Bread Flour</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Additives &amp; Colors</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>14254.55</v>
       </c>
       <c r="E2" t="n">
-        <v>20</v>
+        <v>150</v>
       </c>
       <c r="F2" t="n">
-        <v>80</v>
+        <v>450</v>
       </c>
       <c r="G2" t="n">
-        <v>4</v>
-      </c>
-      <c r="H2" t="n">
-        <v>64</v>
+        <v>3</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -500,30 +500,30 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Baking Powder</t>
+          <t>All-Purpose Flour</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Baking Supplies</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>11630.84</v>
       </c>
       <c r="E3" t="n">
-        <v>25</v>
+        <v>120</v>
       </c>
       <c r="F3" t="n">
-        <v>100</v>
+        <v>380</v>
       </c>
       <c r="G3" t="n">
         <v>3</v>
       </c>
-      <c r="H3" t="n">
-        <v>80</v>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -534,30 +534,30 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Cream of Tartar</t>
+          <t>Cake Flour</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Baking Supplies</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>4480.65</v>
       </c>
       <c r="E4" t="n">
-        <v>10</v>
+        <v>80</v>
       </c>
       <c r="F4" t="n">
-        <v>40</v>
+        <v>240</v>
       </c>
       <c r="G4" t="n">
         <v>4</v>
       </c>
-      <c r="H4" t="n">
-        <v>32</v>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -568,30 +568,30 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Instant Dry Yeast</t>
+          <t>Refined White Sugar</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Baking Supplies</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>12330.92</v>
       </c>
       <c r="E5" t="n">
-        <v>30</v>
+        <v>140</v>
       </c>
       <c r="F5" t="n">
-        <v>120</v>
+        <v>400</v>
       </c>
       <c r="G5" t="n">
-        <v>3</v>
-      </c>
-      <c r="H5" t="n">
-        <v>96</v>
+        <v>2</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -602,30 +602,30 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Cane Vinegar</t>
+          <t>Brown Sugar</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Condiments &amp; Acids</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>3736.7</v>
       </c>
       <c r="E6" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="F6" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="G6" t="n">
-        <v>2</v>
-      </c>
-      <c r="H6" t="n">
-        <v>120</v>
+        <v>3</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -636,30 +636,30 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Soy Sauce</t>
+          <t>Powdered Sugar (Icing)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Condiments &amp; Acids</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1453.92</v>
       </c>
       <c r="E7" t="n">
         <v>50</v>
       </c>
       <c r="F7" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="G7" t="n">
-        <v>2</v>
-      </c>
-      <c r="H7" t="n">
-        <v>160</v>
+        <v>3</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -670,30 +670,30 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Condensed Milk</t>
+          <t>Unsalted Butter</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Dairy</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>9244.059999999999</v>
       </c>
       <c r="E8" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="F8" t="n">
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="G8" t="n">
-        <v>3</v>
-      </c>
-      <c r="H8" t="n">
-        <v>200</v>
+        <v>2</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -704,30 +704,30 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Evaporated Milk</t>
+          <t>Salted Butter</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Dairy</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>3412.01</v>
       </c>
       <c r="E9" t="n">
         <v>50</v>
       </c>
       <c r="F9" t="n">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="G9" t="n">
         <v>2</v>
       </c>
-      <c r="H9" t="n">
-        <v>160</v>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -738,30 +738,30 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Powdered Milk</t>
+          <t>Margarine</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Dairy</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>4701.53</v>
       </c>
       <c r="E10" t="n">
-        <v>45</v>
+        <v>75</v>
       </c>
       <c r="F10" t="n">
-        <v>180</v>
+        <v>250</v>
       </c>
       <c r="G10" t="n">
         <v>3</v>
       </c>
-      <c r="H10" t="n">
-        <v>144</v>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -772,30 +772,30 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Fresh Whole Egg Whites</t>
+          <t>Vegetable Shortening</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Dairy &amp; Eggs</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>4018.2</v>
       </c>
       <c r="E11" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="F11" t="n">
-        <v>160</v>
+        <v>210</v>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H11" t="n">
-        <v>128</v>
+        <v>4</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -806,21 +806,19 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Fresh Whole Eggs</t>
+          <t>Pasteurized Whole Eggs</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Dairy &amp; Eggs</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>18123.44</v>
       </c>
       <c r="E12" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="F12" t="n">
         <v>350</v>
@@ -828,8 +826,10 @@
       <c r="G12" t="n">
         <v>1</v>
       </c>
-      <c r="H12" t="n">
-        <v>280</v>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -840,30 +840,30 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>All-Vegetable Shortening</t>
+          <t>Egg Yolks (Liquid)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Dairy &amp; Fats</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>2657.67</v>
       </c>
       <c r="E13" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="F13" t="n">
-        <v>200</v>
+        <v>140</v>
       </c>
       <c r="G13" t="n">
-        <v>3</v>
-      </c>
-      <c r="H13" t="n">
-        <v>160</v>
+        <v>2</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -874,30 +874,30 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Baking Shortening</t>
+          <t>Egg Whites (Liquid)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Dairy &amp; Fats</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>2328.22</v>
       </c>
       <c r="E14" t="n">
-        <v>55</v>
+        <v>35</v>
       </c>
       <c r="F14" t="n">
-        <v>220</v>
+        <v>120</v>
       </c>
       <c r="G14" t="n">
-        <v>3</v>
-      </c>
-      <c r="H14" t="n">
-        <v>176</v>
+        <v>2</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -908,30 +908,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Salted Creamery Butter</t>
+          <t>Full Cream Milk</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Dairy &amp; Fats</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>8720.33</v>
       </c>
       <c r="E15" t="n">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="F15" t="n">
-        <v>260</v>
+        <v>280</v>
       </c>
       <c r="G15" t="n">
         <v>2</v>
       </c>
-      <c r="H15" t="n">
-        <v>208</v>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -942,30 +942,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Seedless Raisins</t>
+          <t>Skimmed Milk Powder</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Dry Goods</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>1854.72</v>
       </c>
       <c r="E16" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="F16" t="n">
-        <v>80</v>
+        <v>165</v>
       </c>
       <c r="G16" t="n">
         <v>4</v>
       </c>
-      <c r="H16" t="n">
-        <v>64</v>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -976,30 +976,30 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Vanilla Extract</t>
+          <t>Evaporated Milk</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Flavorings &amp; Extracts</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
           <t>L</t>
         </is>
       </c>
+      <c r="D17" t="n">
+        <v>3644.92</v>
+      </c>
       <c r="E17" t="n">
-        <v>8</v>
+        <v>60</v>
       </c>
       <c r="F17" t="n">
-        <v>30</v>
+        <v>190</v>
       </c>
       <c r="G17" t="n">
-        <v>5</v>
-      </c>
-      <c r="H17" t="n">
-        <v>24</v>
+        <v>3</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -1010,30 +1010,30 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>All-Purpose Wheat Flour</t>
+          <t>Condensed Milk</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Grains &amp; Flours</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>4314.33</v>
       </c>
       <c r="E18" t="n">
-        <v>120</v>
+        <v>70</v>
       </c>
       <c r="F18" t="n">
-        <v>500</v>
+        <v>225</v>
       </c>
       <c r="G18" t="n">
         <v>3</v>
       </c>
-      <c r="H18" t="n">
-        <v>400</v>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -1044,30 +1044,30 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Cornstarch</t>
+          <t>Heavy Whipping Cream</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Grains &amp; Flours</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>3259.36</v>
       </c>
       <c r="E19" t="n">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="F19" t="n">
-        <v>140</v>
+        <v>170</v>
       </c>
       <c r="G19" t="n">
-        <v>3</v>
-      </c>
-      <c r="H19" t="n">
-        <v>112</v>
+        <v>2</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -1078,30 +1078,30 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Glutinous Rice (Malagkit for Pinipig)</t>
+          <t>Instant Dry Yeast</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Grains &amp; Flours</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>929.61</v>
       </c>
       <c r="E20" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="F20" t="n">
-        <v>300</v>
+        <v>65</v>
       </c>
       <c r="G20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H20" t="n">
-        <v>240</v>
+        <v>5</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -1112,30 +1112,30 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Hard Wheat Bread Flour</t>
+          <t>Active Dry Yeast</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Grains &amp; Flours</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>405.4</v>
       </c>
       <c r="E21" t="n">
-        <v>150</v>
+        <v>15</v>
       </c>
       <c r="F21" t="n">
-        <v>600</v>
+        <v>40</v>
       </c>
       <c r="G21" t="n">
-        <v>3</v>
-      </c>
-      <c r="H21" t="n">
-        <v>480</v>
+        <v>5</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="22">
@@ -1146,30 +1146,30 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Purified Water</t>
+          <t>Baking Powder (Double Acting)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Liquids</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>971.34</v>
       </c>
       <c r="E22" t="n">
-        <v>200</v>
+        <v>20</v>
       </c>
       <c r="F22" t="n">
-        <v>800</v>
+        <v>70</v>
       </c>
       <c r="G22" t="n">
-        <v>1</v>
-      </c>
-      <c r="H22" t="n">
-        <v>640</v>
+        <v>4</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="23">
@@ -1180,30 +1180,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Cleaned Chicken Crop (Butse)</t>
+          <t>Baking Soda</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Meat &amp; Poultry</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>851.73</v>
       </c>
       <c r="E23" t="n">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="F23" t="n">
-        <v>180</v>
+        <v>55</v>
       </c>
       <c r="G23" t="n">
-        <v>2</v>
-      </c>
-      <c r="H23" t="n">
-        <v>144</v>
+        <v>4</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -1214,30 +1214,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Pork Skin with Back Fat</t>
+          <t>Iodized Fine Salt</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Meat &amp; Poultry</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>1680.72</v>
       </c>
       <c r="E24" t="n">
-        <v>90</v>
+        <v>25</v>
       </c>
       <c r="F24" t="n">
-        <v>400</v>
+        <v>80</v>
       </c>
       <c r="G24" t="n">
-        <v>2</v>
-      </c>
-      <c r="H24" t="n">
-        <v>320</v>
+        <v>3</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -1248,30 +1248,30 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Raw Shelled Peanuts</t>
+          <t>Dark Chocolate Couverture (65%)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Nuts &amp; Seeds</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>4626.33</v>
       </c>
       <c r="E25" t="n">
-        <v>85</v>
+        <v>70</v>
       </c>
       <c r="F25" t="n">
-        <v>380</v>
+        <v>240</v>
       </c>
       <c r="G25" t="n">
-        <v>3</v>
-      </c>
-      <c r="H25" t="n">
-        <v>304</v>
+        <v>5</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="26">
@@ -1282,30 +1282,30 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Toasted Sesame Seeds</t>
+          <t>Milk Chocolate Chips</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Nuts &amp; Seeds</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>3504.36</v>
       </c>
       <c r="E26" t="n">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="F26" t="n">
-        <v>60</v>
+        <v>180</v>
       </c>
       <c r="G26" t="n">
-        <v>3</v>
-      </c>
-      <c r="H26" t="n">
-        <v>48</v>
+        <v>4</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="27">
@@ -1316,30 +1316,30 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Palm Cooking Oil</t>
+          <t>White Chocolate Compound</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Oils &amp; Fats</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>1765.87</v>
       </c>
       <c r="E27" t="n">
-        <v>100</v>
+        <v>45</v>
       </c>
       <c r="F27" t="n">
-        <v>450</v>
+        <v>145</v>
       </c>
       <c r="G27" t="n">
-        <v>2</v>
-      </c>
-      <c r="H27" t="n">
-        <v>360</v>
+        <v>4</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="28">
@@ -1350,30 +1350,30 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Pure Pork Lard</t>
+          <t>Alkalized Cocoa Powder</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Oils &amp; Fats</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>3117.35</v>
       </c>
       <c r="E28" t="n">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="F28" t="n">
-        <v>250</v>
+        <v>155</v>
       </c>
       <c r="G28" t="n">
-        <v>2</v>
-      </c>
-      <c r="H28" t="n">
-        <v>200</v>
+        <v>5</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="29">
@@ -1384,30 +1384,30 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Refined Peanut Oil</t>
+          <t>Pure Vanilla Extract</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Oils &amp; Fats</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
           <t>L</t>
         </is>
       </c>
+      <c r="D29" t="n">
+        <v>385.66</v>
+      </c>
       <c r="E29" t="n">
+        <v>10</v>
+      </c>
+      <c r="F29" t="n">
         <v>35</v>
       </c>
-      <c r="F29" t="n">
-        <v>150</v>
-      </c>
       <c r="G29" t="n">
-        <v>3</v>
-      </c>
-      <c r="H29" t="n">
-        <v>120</v>
+        <v>6</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -1418,30 +1418,30 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Fresh Carrots</t>
+          <t>Artificial Vanilla Flavoring</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Produce / Agricultural</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>835.65</v>
       </c>
       <c r="E30" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="F30" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="G30" t="n">
-        <v>2</v>
-      </c>
-      <c r="H30" t="n">
-        <v>96</v>
+        <v>3</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="31">
@@ -1452,30 +1452,30 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Fresh Cassava Tubers</t>
+          <t>Ube Flavor Paste</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Produce / Agricultural</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>2205.47</v>
       </c>
       <c r="E31" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="F31" t="n">
-        <v>260</v>
+        <v>105</v>
       </c>
       <c r="G31" t="n">
-        <v>2</v>
-      </c>
-      <c r="H31" t="n">
-        <v>208</v>
+        <v>4</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="32">
@@ -1486,30 +1486,30 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Fresh Garlic</t>
+          <t>Pandan Extract Essence</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Produce / Agricultural</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>384.59</v>
       </c>
       <c r="E32" t="n">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F32" t="n">
-        <v>100</v>
+        <v>30</v>
       </c>
       <c r="G32" t="n">
-        <v>2</v>
-      </c>
-      <c r="H32" t="n">
-        <v>80</v>
+        <v>4</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -1520,30 +1520,30 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Fresh Ginger</t>
+          <t>Ground Cinnamon Powder</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Produce / Agricultural</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>505.71</v>
       </c>
       <c r="E33" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F33" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="G33" t="n">
-        <v>2</v>
-      </c>
-      <c r="H33" t="n">
-        <v>64</v>
+        <v>5</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="34">
@@ -1554,30 +1554,30 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Fresh Grated Coconut Meat</t>
+          <t>Nutmeg Powder</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Produce / Agricultural</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>345.49</v>
       </c>
       <c r="E34" t="n">
-        <v>50</v>
+        <v>5</v>
       </c>
       <c r="F34" t="n">
-        <v>220</v>
+        <v>18</v>
       </c>
       <c r="G34" t="n">
-        <v>1</v>
-      </c>
-      <c r="H34" t="n">
-        <v>176</v>
+        <v>6</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="35">
@@ -1588,30 +1588,30 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Fresh Mature Coconut Meat</t>
+          <t>Cheddar Cheese Block</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Produce / Agricultural</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>3523.72</v>
       </c>
       <c r="E35" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="F35" t="n">
-        <v>190</v>
+        <v>175</v>
       </c>
       <c r="G35" t="n">
-        <v>1</v>
-      </c>
-      <c r="H35" t="n">
-        <v>152</v>
+        <v>3</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="36">
@@ -1622,30 +1622,30 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Fresh Purple Yam Tubers</t>
+          <t>Cream Cheese</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Produce / Agricultural</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>6561.04</v>
       </c>
       <c r="E36" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="F36" t="n">
-        <v>170</v>
+        <v>200</v>
       </c>
       <c r="G36" t="n">
         <v>3</v>
       </c>
-      <c r="H36" t="n">
-        <v>136</v>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="37">
@@ -1656,30 +1656,30 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Fresh Sweet Potato</t>
+          <t>Grated Parmesan Cheese</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Produce / Agricultural</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>1130.25</v>
       </c>
       <c r="E37" t="n">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="F37" t="n">
-        <v>180</v>
+        <v>80</v>
       </c>
       <c r="G37" t="n">
-        <v>2</v>
-      </c>
-      <c r="H37" t="n">
-        <v>144</v>
+        <v>4</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="38">
@@ -1690,30 +1690,30 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Green Raw Papaya</t>
+          <t>Quick-Melt Cheese</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Produce / Agricultural</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>3058.33</v>
       </c>
       <c r="E38" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="F38" t="n">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="G38" t="n">
-        <v>2</v>
-      </c>
-      <c r="H38" t="n">
-        <v>112</v>
+        <v>3</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="39">
@@ -1724,30 +1724,30 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Pandan Leaves</t>
+          <t>Roasted Almond Slices</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Produce / Agricultural</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>1257.84</v>
       </c>
       <c r="E39" t="n">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="F39" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="G39" t="n">
-        <v>2</v>
-      </c>
-      <c r="H39" t="n">
-        <v>24</v>
+        <v>6</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="40">
@@ -1758,30 +1758,30 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Red Bell Peppers</t>
+          <t>Walnut Halves</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Produce / Agricultural</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>767.91</v>
       </c>
       <c r="E40" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F40" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="G40" t="n">
-        <v>2</v>
-      </c>
-      <c r="H40" t="n">
-        <v>56</v>
+        <v>6</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="41">
@@ -1792,30 +1792,30 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Red Chili Peppers (Siling Labuyo)</t>
+          <t>Desiccated Coconut (Medium)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Produce / Agricultural</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>1753.34</v>
       </c>
       <c r="E41" t="n">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="F41" t="n">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="G41" t="n">
-        <v>2</v>
-      </c>
-      <c r="H41" t="n">
-        <v>40</v>
+        <v>4</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="42">
@@ -1826,30 +1826,30 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Red Onions</t>
+          <t>Black Sesame Seeds</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Produce / Agricultural</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>545.54</v>
       </c>
       <c r="E42" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="F42" t="n">
-        <v>130</v>
+        <v>45</v>
       </c>
       <c r="G42" t="n">
-        <v>2</v>
-      </c>
-      <c r="H42" t="n">
-        <v>104</v>
+        <v>5</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="43">
@@ -1860,30 +1860,30 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Unripe Green Saba Bananas</t>
+          <t>White Sesame Seeds</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Produce / Agricultural</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>988.76</v>
       </c>
       <c r="E43" t="n">
-        <v>110</v>
+        <v>18</v>
       </c>
       <c r="F43" t="n">
-        <v>480</v>
+        <v>60</v>
       </c>
       <c r="G43" t="n">
-        <v>2</v>
-      </c>
-      <c r="H43" t="n">
-        <v>384</v>
+        <v>4</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="44">
@@ -1894,30 +1894,30 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Fresh Acetes Shrimp (Alamang)</t>
+          <t>Strawberry Jam Filling</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Seafood</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>2753.54</v>
       </c>
       <c r="E44" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="F44" t="n">
-        <v>220</v>
+        <v>130</v>
       </c>
       <c r="G44" t="n">
-        <v>1</v>
-      </c>
-      <c r="H44" t="n">
-        <v>176</v>
+        <v>3</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="45">
@@ -1928,30 +1928,30 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Fresh Bangus (Milkfish) Skin</t>
+          <t>Blueberry Fruit Filling</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Seafood</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>2379.03</v>
       </c>
       <c r="E45" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="F45" t="n">
-        <v>190</v>
+        <v>110</v>
       </c>
       <c r="G45" t="n">
-        <v>2</v>
-      </c>
-      <c r="H45" t="n">
-        <v>152</v>
+        <v>4</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="46">
@@ -1962,30 +1962,30 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Fresh Chiton Mollusk (Kibit)</t>
+          <t>Bavarian Cream Filling</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Seafood</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>5437.78</v>
       </c>
       <c r="E46" t="n">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="F46" t="n">
-        <v>320</v>
+        <v>160</v>
       </c>
       <c r="G46" t="n">
-        <v>1</v>
-      </c>
-      <c r="H46" t="n">
-        <v>256</v>
+        <v>3</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="47">
@@ -1996,30 +1996,30 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Fresh Kabasi Fish</t>
+          <t>Pineapple Crushed (Canned)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Seafood</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>1599.89</v>
       </c>
       <c r="E47" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="F47" t="n">
-        <v>160</v>
+        <v>100</v>
       </c>
       <c r="G47" t="n">
-        <v>1</v>
-      </c>
-      <c r="H47" t="n">
-        <v>128</v>
+        <v>4</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="48">
@@ -2030,30 +2030,30 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Fresh Sapsap Fish</t>
+          <t>Cornstarch (Maizena)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Seafood</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>2976.39</v>
       </c>
       <c r="E48" t="n">
         <v>40</v>
       </c>
       <c r="F48" t="n">
-        <v>170</v>
+        <v>140</v>
       </c>
       <c r="G48" t="n">
-        <v>1</v>
-      </c>
-      <c r="H48" t="n">
-        <v>136</v>
+        <v>3</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="49">
@@ -2064,30 +2064,30 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Cheese Seasoning Powder</t>
+          <t>Bread Improver (Enzyme)</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Seasonings &amp; Powders</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>649.5599999999999</v>
       </c>
       <c r="E49" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="F49" t="n">
-        <v>60</v>
+        <v>26</v>
       </c>
       <c r="G49" t="n">
-        <v>3</v>
-      </c>
-      <c r="H49" t="n">
-        <v>48</v>
+        <v>5</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="50">
@@ -2098,30 +2098,30 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Coarse Rock Salt</t>
+          <t>Emulsifier Paste (Ovalette)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Seasonings / Salts</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>829.7</v>
       </c>
       <c r="E50" t="n">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="F50" t="n">
-        <v>150</v>
+        <v>40</v>
       </c>
       <c r="G50" t="n">
-        <v>3</v>
-      </c>
-      <c r="H50" t="n">
-        <v>120</v>
+        <v>5</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="51">
@@ -2132,30 +2132,30 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Iodized Salt</t>
+          <t>Calcium Propionate (Preservative)</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Seasonings / Salts</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>506.37</v>
       </c>
       <c r="E51" t="n">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="F51" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="G51" t="n">
-        <v>3</v>
-      </c>
-      <c r="H51" t="n">
-        <v>80</v>
+        <v>6</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="52">
@@ -2166,30 +2166,30 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Dried Bay Leaves (Laurel)</t>
+          <t>Liquid Glucose Syrup</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Spices &amp; Seasonings</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>2662.87</v>
       </c>
       <c r="E52" t="n">
-        <v>6</v>
+        <v>35</v>
       </c>
       <c r="F52" t="n">
-        <v>25</v>
+        <v>120</v>
       </c>
       <c r="G52" t="n">
         <v>4</v>
       </c>
-      <c r="H52" t="n">
-        <v>20</v>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="53">
@@ -2200,30 +2200,30 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Dried Red Chili Flakes</t>
+          <t>Honey Pure Bee</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Spices &amp; Seasonings</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>745.36</v>
       </c>
       <c r="E53" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F53" t="n">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="G53" t="n">
-        <v>4</v>
-      </c>
-      <c r="H53" t="n">
-        <v>32</v>
+        <v>5</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="54">
@@ -2234,30 +2234,30 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Garlic Powder</t>
+          <t>Matcha Green Tea Powder</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Spices &amp; Seasonings</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>738.58</v>
       </c>
       <c r="E54" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F54" t="n">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="G54" t="n">
-        <v>4</v>
-      </c>
-      <c r="H54" t="n">
-        <v>48</v>
+        <v>7</v>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="55">
@@ -2268,30 +2268,30 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Ground Black Pepper</t>
+          <t>Red Food Coloring (Gel)</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Spices &amp; Seasonings</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>473.8</v>
       </c>
       <c r="E55" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="F55" t="n">
-        <v>50</v>
+        <v>14</v>
       </c>
       <c r="G55" t="n">
         <v>4</v>
       </c>
-      <c r="H55" t="n">
-        <v>40</v>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="56">
@@ -2302,30 +2302,30 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>White Pepper Powder</t>
+          <t>Yellow Food Coloring (Gel)</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Spices &amp; Seasonings</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>514.25</v>
       </c>
       <c r="E56" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="F56" t="n">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="G56" t="n">
         <v>4</v>
       </c>
-      <c r="H56" t="n">
-        <v>32</v>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="57">
@@ -2336,30 +2336,30 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Whole Black Peppercorns</t>
+          <t>Green Food Coloring (Gel)</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Spices &amp; Seasonings</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>522.09</v>
       </c>
       <c r="E57" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="F57" t="n">
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="G57" t="n">
         <v>4</v>
       </c>
-      <c r="H57" t="n">
-        <v>48</v>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="58">
@@ -2370,30 +2370,30 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Muscovado Brown Sugar</t>
+          <t>Instant Coffee Powder</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Sweeteners</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>1048.59</v>
       </c>
       <c r="E58" t="n">
+        <v>18</v>
+      </c>
+      <c r="F58" t="n">
         <v>55</v>
       </c>
-      <c r="F58" t="n">
-        <v>240</v>
-      </c>
       <c r="G58" t="n">
-        <v>3</v>
-      </c>
-      <c r="H58" t="n">
-        <v>192</v>
+        <v>4</v>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="59">
@@ -2404,30 +2404,30 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Panutsa Cane Sugar</t>
+          <t>Rolled Oats (Old Fashioned)</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Sweeteners</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>1392.24</v>
       </c>
       <c r="E59" t="n">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="F59" t="n">
-        <v>190</v>
+        <v>85</v>
       </c>
       <c r="G59" t="n">
-        <v>3</v>
-      </c>
-      <c r="H59" t="n">
-        <v>152</v>
+        <v>4</v>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
     <row r="60">
@@ -2438,30 +2438,30 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Refined White Sugar</t>
+          <t>Golden Raisins Seedless</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Sweeteners</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>1285.57</v>
       </c>
       <c r="E60" t="n">
-        <v>110</v>
+        <v>22</v>
       </c>
       <c r="F60" t="n">
-        <v>480</v>
+        <v>75</v>
       </c>
       <c r="G60" t="n">
-        <v>2</v>
-      </c>
-      <c r="H60" t="n">
-        <v>384</v>
+        <v>5</v>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(dataset): calibrate dataset to 45% received / 55% consumed to showcase realistic usage strain and shortage alerts
</commit_message>
<xml_diff>
--- a/RMIMS_59_RAW_MATERIALS_CATALOG.xlsx
+++ b/RMIMS_59_RAW_MATERIALS_CATALOG.xlsx
@@ -475,20 +475,20 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>14254.55</v>
+        <v>150</v>
       </c>
       <c r="E2" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="F2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="G2" t="n">
         <v>3</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -509,20 +509,20 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>11630.84</v>
+        <v>193</v>
       </c>
       <c r="E3" t="n">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="F3" t="n">
-        <v>380</v>
+        <v>350</v>
       </c>
       <c r="G3" t="n">
         <v>3</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>STABLE</t>
         </is>
       </c>
     </row>
@@ -543,20 +543,20 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>4480.65</v>
+        <v>27</v>
       </c>
       <c r="E4" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="F4" t="n">
-        <v>240</v>
+        <v>220</v>
       </c>
       <c r="G4" t="n">
         <v>4</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>OUT OF STOCK</t>
         </is>
       </c>
     </row>
@@ -577,20 +577,20 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>12330.92</v>
+        <v>138</v>
       </c>
       <c r="E5" t="n">
-        <v>140</v>
+        <v>180</v>
       </c>
       <c r="F5" t="n">
-        <v>400</v>
+        <v>380</v>
       </c>
       <c r="G5" t="n">
         <v>2</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -611,13 +611,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>3736.7</v>
+        <v>172</v>
       </c>
       <c r="E6" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="F6" t="n">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="G6" t="n">
         <v>3</v>
@@ -645,20 +645,20 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1453.92</v>
+        <v>15</v>
       </c>
       <c r="E7" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="F7" t="n">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="G7" t="n">
         <v>3</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>OUT OF STOCK</t>
         </is>
       </c>
     </row>
@@ -679,20 +679,20 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>9244.059999999999</v>
+        <v>90</v>
       </c>
       <c r="E8" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="F8" t="n">
-        <v>300</v>
+        <v>280</v>
       </c>
       <c r="G8" t="n">
         <v>2</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -713,20 +713,20 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>3412.01</v>
+        <v>91</v>
       </c>
       <c r="E9" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="F9" t="n">
-        <v>180</v>
+        <v>160</v>
       </c>
       <c r="G9" t="n">
         <v>2</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>STABLE</t>
         </is>
       </c>
     </row>
@@ -747,13 +747,13 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>4701.53</v>
+        <v>197</v>
       </c>
       <c r="E10" t="n">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="F10" t="n">
-        <v>250</v>
+        <v>230</v>
       </c>
       <c r="G10" t="n">
         <v>3</v>
@@ -781,20 +781,20 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>4018.2</v>
+        <v>24</v>
       </c>
       <c r="E11" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="F11" t="n">
-        <v>210</v>
+        <v>190</v>
       </c>
       <c r="G11" t="n">
         <v>4</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>OUT OF STOCK</t>
         </is>
       </c>
     </row>
@@ -815,20 +815,20 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>18123.44</v>
+        <v>102</v>
       </c>
       <c r="E12" t="n">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="F12" t="n">
-        <v>350</v>
+        <v>320</v>
       </c>
       <c r="G12" t="n">
         <v>1</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -849,20 +849,20 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>2657.67</v>
+        <v>63</v>
       </c>
       <c r="E13" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="F13" t="n">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="G13" t="n">
         <v>2</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>STABLE</t>
         </is>
       </c>
     </row>
@@ -883,20 +883,20 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>2328.22</v>
+        <v>13</v>
       </c>
       <c r="E14" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="F14" t="n">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="G14" t="n">
         <v>2</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>OUT OF STOCK</t>
         </is>
       </c>
     </row>
@@ -917,20 +917,20 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>8720.33</v>
+        <v>76</v>
       </c>
       <c r="E15" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="F15" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="G15" t="n">
         <v>2</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -951,13 +951,13 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1854.72</v>
+        <v>130</v>
       </c>
       <c r="E16" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="F16" t="n">
-        <v>165</v>
+        <v>150</v>
       </c>
       <c r="G16" t="n">
         <v>4</v>
@@ -985,20 +985,20 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>3644.92</v>
+        <v>91</v>
       </c>
       <c r="E17" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F17" t="n">
-        <v>190</v>
+        <v>170</v>
       </c>
       <c r="G17" t="n">
         <v>3</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>STABLE</t>
         </is>
       </c>
     </row>
@@ -1019,20 +1019,20 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>4314.33</v>
+        <v>64</v>
       </c>
       <c r="E18" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="F18" t="n">
-        <v>225</v>
+        <v>200</v>
       </c>
       <c r="G18" t="n">
         <v>3</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -1053,20 +1053,20 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>3259.36</v>
+        <v>18</v>
       </c>
       <c r="E19" t="n">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="F19" t="n">
-        <v>170</v>
+        <v>150</v>
       </c>
       <c r="G19" t="n">
         <v>2</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>OUT OF STOCK</t>
         </is>
       </c>
     </row>
@@ -1087,20 +1087,20 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>929.61</v>
+        <v>19</v>
       </c>
       <c r="E20" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F20" t="n">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="G20" t="n">
         <v>5</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -1121,20 +1121,20 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>405.4</v>
+        <v>25</v>
       </c>
       <c r="E21" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F21" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="G21" t="n">
         <v>5</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>STABLE</t>
         </is>
       </c>
     </row>
@@ -1155,13 +1155,13 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>971.34</v>
+        <v>53</v>
       </c>
       <c r="E22" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F22" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="G22" t="n">
         <v>4</v>
@@ -1189,20 +1189,20 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>851.73</v>
+        <v>6</v>
       </c>
       <c r="E23" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F23" t="n">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="G23" t="n">
         <v>4</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>OUT OF STOCK</t>
         </is>
       </c>
     </row>
@@ -1223,13 +1223,13 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>1680.72</v>
+        <v>65</v>
       </c>
       <c r="E24" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F24" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="G24" t="n">
         <v>3</v>
@@ -1257,20 +1257,20 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>4626.33</v>
+        <v>73</v>
       </c>
       <c r="E25" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="F25" t="n">
-        <v>240</v>
+        <v>210</v>
       </c>
       <c r="G25" t="n">
         <v>5</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -1291,20 +1291,20 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>3504.36</v>
+        <v>84</v>
       </c>
       <c r="E26" t="n">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="F26" t="n">
-        <v>180</v>
+        <v>160</v>
       </c>
       <c r="G26" t="n">
         <v>4</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>STABLE</t>
         </is>
       </c>
     </row>
@@ -1325,20 +1325,20 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>1765.87</v>
+        <v>14</v>
       </c>
       <c r="E27" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="F27" t="n">
-        <v>145</v>
+        <v>130</v>
       </c>
       <c r="G27" t="n">
         <v>4</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>OUT OF STOCK</t>
         </is>
       </c>
     </row>
@@ -1359,20 +1359,20 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>3117.35</v>
+        <v>43</v>
       </c>
       <c r="E28" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="F28" t="n">
-        <v>155</v>
+        <v>135</v>
       </c>
       <c r="G28" t="n">
         <v>5</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -1393,13 +1393,13 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>385.66</v>
+        <v>32</v>
       </c>
       <c r="E29" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F29" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="G29" t="n">
         <v>6</v>
@@ -1427,20 +1427,20 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>835.65</v>
+        <v>26</v>
       </c>
       <c r="E30" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F30" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="G30" t="n">
         <v>3</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>STABLE</t>
         </is>
       </c>
     </row>
@@ -1461,20 +1461,20 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>2205.47</v>
+        <v>35</v>
       </c>
       <c r="E31" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="F31" t="n">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="G31" t="n">
         <v>4</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -1495,20 +1495,20 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>384.59</v>
+        <v>3</v>
       </c>
       <c r="E32" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F32" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G32" t="n">
         <v>4</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>OUT OF STOCK</t>
         </is>
       </c>
     </row>
@@ -1529,13 +1529,13 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>505.71</v>
+        <v>25</v>
       </c>
       <c r="E33" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F33" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="G33" t="n">
         <v>5</v>
@@ -1563,13 +1563,13 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>345.49</v>
+        <v>15</v>
       </c>
       <c r="E34" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F34" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="G34" t="n">
         <v>6</v>
@@ -1597,20 +1597,20 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>3523.72</v>
+        <v>52</v>
       </c>
       <c r="E35" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="F35" t="n">
-        <v>175</v>
+        <v>155</v>
       </c>
       <c r="G35" t="n">
         <v>3</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -1631,20 +1631,20 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>6561.04</v>
+        <v>23</v>
       </c>
       <c r="E36" t="n">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="F36" t="n">
-        <v>200</v>
+        <v>175</v>
       </c>
       <c r="G36" t="n">
         <v>3</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>OUT OF STOCK</t>
         </is>
       </c>
     </row>
@@ -1665,20 +1665,20 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1130.25</v>
+        <v>39</v>
       </c>
       <c r="E37" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F37" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="G37" t="n">
         <v>4</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>STABLE</t>
         </is>
       </c>
     </row>
@@ -1699,13 +1699,13 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>3058.33</v>
+        <v>122</v>
       </c>
       <c r="E38" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="F38" t="n">
-        <v>150</v>
+        <v>130</v>
       </c>
       <c r="G38" t="n">
         <v>3</v>
@@ -1733,20 +1733,20 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>1257.84</v>
+        <v>24</v>
       </c>
       <c r="E39" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F39" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="G39" t="n">
         <v>6</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -1767,20 +1767,20 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>767.91</v>
+        <v>9</v>
       </c>
       <c r="E40" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F40" t="n">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="G40" t="n">
         <v>6</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>OUT OF STOCK</t>
         </is>
       </c>
     </row>
@@ -1801,20 +1801,20 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>1753.34</v>
+        <v>61</v>
       </c>
       <c r="E41" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="F41" t="n">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="G41" t="n">
         <v>4</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>STABLE</t>
         </is>
       </c>
     </row>
@@ -1835,13 +1835,13 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>545.54</v>
+        <v>38</v>
       </c>
       <c r="E42" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F42" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G42" t="n">
         <v>5</v>
@@ -1869,20 +1869,20 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>988.76</v>
+        <v>22</v>
       </c>
       <c r="E43" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F43" t="n">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="G43" t="n">
         <v>4</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -1903,20 +1903,20 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>2753.54</v>
+        <v>15</v>
       </c>
       <c r="E44" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="F44" t="n">
-        <v>130</v>
+        <v>115</v>
       </c>
       <c r="G44" t="n">
         <v>3</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>OUT OF STOCK</t>
         </is>
       </c>
     </row>
@@ -1937,20 +1937,20 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>2379.03</v>
+        <v>51</v>
       </c>
       <c r="E45" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="F45" t="n">
-        <v>110</v>
+        <v>95</v>
       </c>
       <c r="G45" t="n">
         <v>4</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>STABLE</t>
         </is>
       </c>
     </row>
@@ -1971,20 +1971,20 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>5437.78</v>
+        <v>47</v>
       </c>
       <c r="E46" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="F46" t="n">
-        <v>160</v>
+        <v>140</v>
       </c>
       <c r="G46" t="n">
         <v>3</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -2005,13 +2005,13 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>1599.89</v>
+        <v>79</v>
       </c>
       <c r="E47" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="F47" t="n">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="G47" t="n">
         <v>4</v>
@@ -2039,20 +2039,20 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>2976.39</v>
+        <v>66</v>
       </c>
       <c r="E48" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="F48" t="n">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="G48" t="n">
         <v>3</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>STABLE</t>
         </is>
       </c>
     </row>
@@ -2073,20 +2073,20 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>649.5599999999999</v>
+        <v>5</v>
       </c>
       <c r="E49" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F49" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="G49" t="n">
         <v>5</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>OUT OF STOCK</t>
         </is>
       </c>
     </row>
@@ -2107,20 +2107,20 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>829.7</v>
+        <v>11</v>
       </c>
       <c r="E50" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F50" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="G50" t="n">
         <v>5</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -2141,13 +2141,13 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>506.37</v>
+        <v>26</v>
       </c>
       <c r="E51" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F51" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G51" t="n">
         <v>6</v>
@@ -2175,20 +2175,20 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>2662.87</v>
+        <v>56</v>
       </c>
       <c r="E52" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="F52" t="n">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="G52" t="n">
         <v>4</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>STABLE</t>
         </is>
       </c>
     </row>
@@ -2209,20 +2209,20 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>745.36</v>
+        <v>7</v>
       </c>
       <c r="E53" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F53" t="n">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="G53" t="n">
         <v>5</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>OUT OF STOCK</t>
         </is>
       </c>
     </row>
@@ -2243,20 +2243,20 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>738.58</v>
+        <v>15</v>
       </c>
       <c r="E54" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F54" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="G54" t="n">
         <v>7</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -2277,13 +2277,13 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>473.8</v>
+        <v>14</v>
       </c>
       <c r="E55" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F55" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G55" t="n">
         <v>4</v>
@@ -2311,13 +2311,13 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>514.25</v>
+        <v>12</v>
       </c>
       <c r="E56" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F56" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G56" t="n">
         <v>4</v>
@@ -2345,20 +2345,20 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>522.09</v>
+        <v>1</v>
       </c>
       <c r="E57" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F57" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G57" t="n">
         <v>4</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>OUT OF STOCK</t>
         </is>
       </c>
     </row>
@@ -2379,20 +2379,20 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>1048.59</v>
+        <v>19</v>
       </c>
       <c r="E58" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F58" t="n">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="G58" t="n">
         <v>4</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -2413,13 +2413,13 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>1392.24</v>
+        <v>70</v>
       </c>
       <c r="E59" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F59" t="n">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="G59" t="n">
         <v>4</v>
@@ -2447,20 +2447,20 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>1285.57</v>
+        <v>36</v>
       </c>
       <c r="E60" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="F60" t="n">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="G60" t="n">
         <v>5</v>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>IN STOCK</t>
+          <t>STABLE</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(dataset): configure situational stock health strictly to Low Stock and Good (0 Out of Stock)
</commit_message>
<xml_diff>
--- a/RMIMS_59_RAW_MATERIALS_CATALOG.xlsx
+++ b/RMIMS_59_RAW_MATERIALS_CATALOG.xlsx
@@ -475,7 +475,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="E2" t="n">
         <v>200</v>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>193</v>
+        <v>345</v>
       </c>
       <c r="E3" t="n">
         <v>160</v>
@@ -522,7 +522,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>STABLE</t>
+          <t>IN STOCK</t>
         </is>
       </c>
     </row>
@@ -543,7 +543,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>27</v>
+        <v>74</v>
       </c>
       <c r="E4" t="n">
         <v>100</v>
@@ -556,7 +556,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>OUT OF STOCK</t>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -577,7 +577,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="E5" t="n">
         <v>180</v>
@@ -611,7 +611,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="E6" t="n">
         <v>80</v>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="E7" t="n">
         <v>60</v>
@@ -658,7 +658,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>OUT OF STOCK</t>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -679,7 +679,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="E8" t="n">
         <v>120</v>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>91</v>
+        <v>158</v>
       </c>
       <c r="E9" t="n">
         <v>70</v>
@@ -726,7 +726,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>STABLE</t>
+          <t>IN STOCK</t>
         </is>
       </c>
     </row>
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="E10" t="n">
         <v>90</v>
@@ -781,7 +781,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>24</v>
+        <v>62</v>
       </c>
       <c r="E11" t="n">
         <v>80</v>
@@ -794,7 +794,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>OUT OF STOCK</t>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -815,7 +815,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="E12" t="n">
         <v>130</v>
@@ -849,7 +849,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>63</v>
+        <v>111</v>
       </c>
       <c r="E13" t="n">
         <v>50</v>
@@ -862,7 +862,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>STABLE</t>
+          <t>IN STOCK</t>
         </is>
       </c>
     </row>
@@ -883,7 +883,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="E14" t="n">
         <v>45</v>
@@ -896,7 +896,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>OUT OF STOCK</t>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -917,7 +917,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E15" t="n">
         <v>100</v>
@@ -951,7 +951,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="E16" t="n">
         <v>60</v>
@@ -985,7 +985,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>91</v>
+        <v>158</v>
       </c>
       <c r="E17" t="n">
         <v>70</v>
@@ -998,7 +998,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>STABLE</t>
+          <t>IN STOCK</t>
         </is>
       </c>
     </row>
@@ -1019,7 +1019,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="E18" t="n">
         <v>80</v>
@@ -1053,7 +1053,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>18</v>
+        <v>49</v>
       </c>
       <c r="E19" t="n">
         <v>65</v>
@@ -1066,7 +1066,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>OUT OF STOCK</t>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -1087,7 +1087,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E20" t="n">
         <v>25</v>
@@ -1121,7 +1121,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="E21" t="n">
         <v>18</v>
@@ -1134,7 +1134,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>STABLE</t>
+          <t>IN STOCK</t>
         </is>
       </c>
     </row>
@@ -1155,7 +1155,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="E22" t="n">
         <v>25</v>
@@ -1189,7 +1189,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E23" t="n">
         <v>20</v>
@@ -1202,7 +1202,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>OUT OF STOCK</t>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -1223,7 +1223,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="E24" t="n">
         <v>30</v>
@@ -1257,7 +1257,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="E25" t="n">
         <v>90</v>
@@ -1291,7 +1291,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>84</v>
+        <v>151</v>
       </c>
       <c r="E26" t="n">
         <v>70</v>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>STABLE</t>
+          <t>IN STOCK</t>
         </is>
       </c>
     </row>
@@ -1325,7 +1325,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="E27" t="n">
         <v>55</v>
@@ -1338,7 +1338,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>OUT OF STOCK</t>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -1359,7 +1359,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E28" t="n">
         <v>55</v>
@@ -1393,7 +1393,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E29" t="n">
         <v>12</v>
@@ -1427,7 +1427,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>26</v>
+        <v>43</v>
       </c>
       <c r="E30" t="n">
         <v>18</v>
@@ -1440,7 +1440,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>STABLE</t>
+          <t>IN STOCK</t>
         </is>
       </c>
     </row>
@@ -1461,7 +1461,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E31" t="n">
         <v>40</v>
@@ -1495,7 +1495,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E32" t="n">
         <v>12</v>
@@ -1508,7 +1508,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>OUT OF STOCK</t>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -1529,7 +1529,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="E33" t="n">
         <v>15</v>
@@ -1563,7 +1563,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E34" t="n">
         <v>6</v>
@@ -1597,7 +1597,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E35" t="n">
         <v>65</v>
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>23</v>
+        <v>58</v>
       </c>
       <c r="E36" t="n">
         <v>75</v>
@@ -1644,7 +1644,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>OUT OF STOCK</t>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -1665,7 +1665,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>39</v>
+        <v>68</v>
       </c>
       <c r="E37" t="n">
         <v>30</v>
@@ -1678,7 +1678,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>STABLE</t>
+          <t>IN STOCK</t>
         </is>
       </c>
     </row>
@@ -1767,7 +1767,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="E40" t="n">
         <v>25</v>
@@ -1780,7 +1780,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>OUT OF STOCK</t>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -1801,7 +1801,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>61</v>
+        <v>104</v>
       </c>
       <c r="E41" t="n">
         <v>45</v>
@@ -1814,7 +1814,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>STABLE</t>
+          <t>IN STOCK</t>
         </is>
       </c>
     </row>
@@ -1835,7 +1835,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E42" t="n">
         <v>18</v>
@@ -1869,7 +1869,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="E43" t="n">
         <v>22</v>
@@ -1903,7 +1903,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="E44" t="n">
         <v>50</v>
@@ -1916,7 +1916,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>OUT OF STOCK</t>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -1937,7 +1937,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>51</v>
+        <v>89</v>
       </c>
       <c r="E45" t="n">
         <v>40</v>
@@ -1950,7 +1950,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>STABLE</t>
+          <t>IN STOCK</t>
         </is>
       </c>
     </row>
@@ -2005,7 +2005,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E47" t="n">
         <v>35</v>
@@ -2039,7 +2039,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>66</v>
+        <v>114</v>
       </c>
       <c r="E48" t="n">
         <v>50</v>
@@ -2052,7 +2052,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>STABLE</t>
+          <t>IN STOCK</t>
         </is>
       </c>
     </row>
@@ -2073,7 +2073,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E49" t="n">
         <v>10</v>
@@ -2086,7 +2086,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>OUT OF STOCK</t>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -2107,7 +2107,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E50" t="n">
         <v>15</v>
@@ -2141,7 +2141,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E51" t="n">
         <v>8</v>
@@ -2175,7 +2175,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>56</v>
+        <v>99</v>
       </c>
       <c r="E52" t="n">
         <v>45</v>
@@ -2188,7 +2188,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>STABLE</t>
+          <t>IN STOCK</t>
         </is>
       </c>
     </row>
@@ -2209,7 +2209,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="E53" t="n">
         <v>25</v>
@@ -2222,7 +2222,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>OUT OF STOCK</t>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -2243,7 +2243,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E54" t="n">
         <v>15</v>
@@ -2277,7 +2277,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E55" t="n">
         <v>5</v>
@@ -2311,7 +2311,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="E56" t="n">
         <v>5</v>
@@ -2345,7 +2345,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E57" t="n">
         <v>4</v>
@@ -2358,7 +2358,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>OUT OF STOCK</t>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -2379,7 +2379,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E58" t="n">
         <v>22</v>
@@ -2413,7 +2413,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="E59" t="n">
         <v>30</v>
@@ -2447,7 +2447,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>36</v>
+        <v>62</v>
       </c>
       <c r="E60" t="n">
         <v>28</v>
@@ -2460,7 +2460,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>STABLE</t>
+          <t>IN STOCK</t>
         </is>
       </c>
     </row>

</xml_diff>